<commit_message>
Commit before modifying main
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -5,34 +5,57 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abish\OneDrive\Desktop\CAPGEMINI-SPRINT\PetstoreAutomationTesting\PetStoreAPIAutomation\src\test\resources\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abish\OneDrive\Desktop\CAPGEMINI-SPRINT\PetstoreAutomationTesting\StoreModule\PetStoreAPITesting\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{77418256-B56F-4272-A57A-8996DC9B3D79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD288F7-0267-4FA5-A78F-7782CF571573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{BB31F1E5-A51E-4CF1-9366-85B0A5AC9C0A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BB31F1E5-A51E-4CF1-9366-85B0A5AC9C0A}"/>
   </bookViews>
   <sheets>
     <sheet name="PetModule" sheetId="1" r:id="rId1"/>
     <sheet name="StoreModule" sheetId="2" r:id="rId2"/>
     <sheet name="UserModule" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>petId</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>shipDate</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>complete</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>sold</t>
+  </si>
+  <si>
+    <t>2026-04-18T08:00:00.000Z</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -66,8 +89,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -391,9 +415,53 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16C93E48-DDC5-465B-BFBF-BA61A801DCAD}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="6" max="6" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>10001</v>
+      </c>
+      <c r="B2">
+        <v>1001</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Implemented DDT and Request Chaining using .xslx file
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abish\OneDrive\Desktop\CAPGEMINI-SPRINT\PetstoreAutomationTesting\StoreModule\PetStoreAPITesting\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD288F7-0267-4FA5-A78F-7782CF571573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64718AB7-B5BE-4A72-915B-B217D5037040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BB31F1E5-A51E-4CF1-9366-85B0A5AC9C0A}"/>
+    <workbookView xWindow="5592" yWindow="3360" windowWidth="17448" windowHeight="8880" activeTab="1" xr2:uid="{BB31F1E5-A51E-4CF1-9366-85B0A5AC9C0A}"/>
   </bookViews>
   <sheets>
     <sheet name="PetModule" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="21">
   <si>
     <t>id</t>
   </si>
@@ -50,10 +50,46 @@
     <t>true</t>
   </si>
   <si>
-    <t>sold</t>
-  </si>
-  <si>
     <t>2026-04-18T08:00:00.000Z</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>placed</t>
+  </si>
+  <si>
+    <t>2026-04-18T09:00:00.000Z</t>
+  </si>
+  <si>
+    <t>approved</t>
+  </si>
+  <si>
+    <t>2026-04-18T10:00:00.000Z</t>
+  </si>
+  <si>
+    <t>delivered</t>
+  </si>
+  <si>
+    <t>2026-04-19T11:30:00.000Z</t>
+  </si>
+  <si>
+    <t>2026-04-20T12:15:00.000Z</t>
+  </si>
+  <si>
+    <t>2026-04-21T09:45:00.000Z</t>
+  </si>
+  <si>
+    <t>2026-04-22T14:20:00.000Z</t>
+  </si>
+  <si>
+    <t>2026-04-23T16:00:00.000Z</t>
+  </si>
+  <si>
+    <t>2026-04-24T11:10:00.000Z</t>
+  </si>
+  <si>
+    <t>2026-04-25T13:50:00.000Z</t>
   </si>
 </sst>
 </file>
@@ -415,9 +451,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16C93E48-DDC5-465B-BFBF-BA61A801DCAD}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="2" width="8.88671875" customWidth="1"/>
     <col min="6" max="6" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
@@ -452,13 +489,193 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>10002</v>
+      </c>
+      <c r="B3">
+        <v>1002</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>10003</v>
+      </c>
+      <c r="B4">
+        <v>1003</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>10004</v>
+      </c>
+      <c r="B5">
+        <v>1004</v>
+      </c>
+      <c r="C5">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>10005</v>
+      </c>
+      <c r="B6">
+        <v>1005</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>10006</v>
+      </c>
+      <c r="B7">
+        <v>1006</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>10007</v>
+      </c>
+      <c r="B8">
+        <v>1007</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>10008</v>
+      </c>
+      <c r="B9">
+        <v>1008</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>10009</v>
+      </c>
+      <c r="B10">
+        <v>1009</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10010</v>
+      </c>
+      <c r="B11">
+        <v>1010</v>
+      </c>
+      <c r="C11">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
achiving ddt using scenario outline and request chaining
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Desktop\petModule\newPet\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193811EC-5B45-4B89-BDCD-1BA18E11924F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6706D974-2386-45C2-A693-AFC312F3E532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3270" yWindow="1035" windowWidth="15375" windowHeight="7785" xr2:uid="{BB31F1E5-A51E-4CF1-9366-85B0A5AC9C0A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{BB31F1E5-A51E-4CF1-9366-85B0A5AC9C0A}"/>
   </bookViews>
   <sheets>
     <sheet name="PetModule" sheetId="1" r:id="rId1"/>
@@ -36,56 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
-  <si>
-    <t>TestCase</t>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>TC_PET_01</t>
-  </si>
-  <si>
-    <t>doggie</t>
-  </si>
-  <si>
-    <t>available</t>
-  </si>
-  <si>
-    <t>TC_PET_02</t>
-  </si>
-  <si>
-    <t>cat</t>
-  </si>
-  <si>
-    <t>TC_PET_03</t>
-  </si>
-  <si>
-    <t>doggie_updated</t>
-  </si>
-  <si>
-    <t>sold</t>
-  </si>
-  <si>
-    <t>TC_PET_07</t>
-  </si>
-  <si>
-    <t>TC_PET_08</t>
-  </si>
-  <si>
-    <t>TC_PET_09</t>
-  </si>
-  <si>
-    <t>invalid</t>
-  </si>
-</sst>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -458,94 +409,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2">
-        <v>2001</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="2">
-        <v>2002</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="2">
-        <v>2001</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2">
-        <v>3001</v>
-      </c>
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="2">
-        <v>0</v>
-      </c>
-      <c r="C7" s="2">
-        <v>123</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Changing Store Module and Implement Scenario Outline
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -3,14 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adithya\Desktop\PetStoreAPITesting\src\test\resources\testData\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1053A3-CE66-4B33-94E9-44D21936163D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{60A97C94-12F1-4EA6-AC86-3D85A9E8B094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{BB31F1E5-A51E-4CF1-9366-85B0A5AC9C0A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BB31F1E5-A51E-4CF1-9366-85B0A5AC9C0A}"/>
   </bookViews>
   <sheets>
     <sheet name="PetModule" sheetId="1" r:id="rId1"/>
@@ -18,6 +13,7 @@
     <sheet name="UserModule" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1:N27"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>

<commit_message>
implement data table and scenario outline
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{60A97C94-12F1-4EA6-AC86-3D85A9E8B094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a8db6bb4be0bfad/Desktop/Pet-Module/PetStore-API/petstore/src/test/resources/testData/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:801_{60A97C94-12F1-4EA6-AC86-3D85A9E8B094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC1BB573-F5EC-4937-8151-95F2E1DAEA8D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BB31F1E5-A51E-4CF1-9366-85B0A5AC9C0A}"/>
+    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7260" xr2:uid="{BB31F1E5-A51E-4CF1-9366-85B0A5AC9C0A}"/>
   </bookViews>
   <sheets>
     <sheet name="PetModule" sheetId="1" r:id="rId1"/>
@@ -13,7 +18,6 @@
     <sheet name="UserModule" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:N27"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="43">
   <si>
     <t>id</t>
   </si>
@@ -140,6 +144,18 @@
   </si>
   <si>
     <t>horse</t>
+  </si>
+  <si>
+    <t>tommy</t>
+  </si>
+  <si>
+    <t>jack</t>
+  </si>
+  <si>
+    <t>puppy</t>
+  </si>
+  <si>
+    <t>pending</t>
   </si>
 </sst>
 </file>
@@ -181,10 +197,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,11 +516,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAAF3744-07D1-4C69-B0DF-3D79C5195282}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.7265625" style="3"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -513,8 +533,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
         <v>1001</v>
       </c>
       <c r="B2" t="s">
@@ -524,8 +544,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
         <v>1003</v>
       </c>
       <c r="B3" t="s">
@@ -535,14 +555,47 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
         <v>1004</v>
       </c>
       <c r="B4" t="s">
         <v>38</v>
       </c>
       <c r="C4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="3">
+        <v>1002</v>
+      </c>
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="3">
+        <v>1005</v>
+      </c>
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>1006</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
         <v>37</v>
       </c>
     </row>
@@ -554,13 +607,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16C93E48-DDC5-465B-BFBF-BA61A801DCAD}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="8.88671875" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="1"/>
+    <col min="1" max="2" width="8.90625" customWidth="1"/>
+    <col min="6" max="6" width="8.90625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -580,7 +633,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>10001</v>
       </c>
@@ -600,7 +653,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>10002</v>
       </c>
@@ -620,7 +673,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>10003</v>
       </c>
@@ -640,7 +693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>10004</v>
       </c>
@@ -660,7 +713,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>10005</v>
       </c>
@@ -680,7 +733,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>10006</v>
       </c>
@@ -700,7 +753,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>10007</v>
       </c>
@@ -720,7 +773,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>10008</v>
       </c>
@@ -740,7 +793,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>10009</v>
       </c>
@@ -760,7 +813,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10010</v>
       </c>
@@ -788,14 +841,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{147E4B78-4D93-4DA5-A9CD-1A53DF8932CE}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -821,7 +874,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1001</v>
       </c>

</xml_diff>